<commit_message>
Accept Mission AW-20260903-003 and reconcile QA
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R8dd4ba551a244856"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R0f61bd7841d94a9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="Ra4228be1d7a246c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R7fa8e4a562f5486d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R0233a0f9577f4b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R58c1d4056dc947d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1078,6 +1078,23 @@
         <x:v>ACCEPTED — described production state not found; QA-CAND-002 closed</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="135" customHeight="1">
+      <x:c r="A21" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B21" s="9" t="str">
+        <x:v>Mission AW-20260903-003 — For Organizations production migration</x:v>
+      </x:c>
+      <x:c r="C21" s="9" t="str">
+        <x:v>Codex independently reviewed commit 6dfb15d from the exact issuance parent 315f8c5. Scope stayed within the four authorized implementation paths plus claude-return.md. The generated Organizations page uses the shared shell, preserves the approved nine-section narrative and honest not-yet-launched framing, includes the four-ring Value/Knowledge/Teams/People landscape, and keeps the two closing actions distinct (mailto for the Organizations-specific invitation; /contact/ for general contact). Full checked-in suites passed 9/9 in root mode and 9/9 with BASE_PATH=/alaya-crafts-website. Desktop 1440px and mobile 390px rendered captures were reviewed for hierarchy, spacing, diagram integrity, contact distinction, and responsive reflow.</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="str">
+        <x:v>0 new — no blocking or corrective findings</x:v>
+      </x:c>
+      <x:c r="E21" s="9" t="str">
+        <x:v>ACCEPTED — For Organizations clears its page-specific Production Reference Gate; no push, merge, deployment, or broader product approval implied</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2267,7 +2284,32 @@
         <x:v>Closed 2026-09-03 by Codex disposition of AW-20260903-002. CIE studies contain the label as non-interactive spans; production instead uses #understanding and ../. The origin of the tracker’s #main combination remains unproved, so no causal explanation is asserted.</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="18" customHeight="1"/>
+    <x:row r="29" ht="135" customHeight="1">
+      <x:c r="A29" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B29" s="9" t="str">
+        <x:v>Production / For Organizations migration</x:v>
+      </x:c>
+      <x:c r="C29" s="9" t="str">
+        <x:v>src/pages/organizations.mjs + src/assets/organizations.css + generated dist/for-organizations/index.html</x:v>
+      </x:c>
+      <x:c r="D29" s="9" t="str">
+        <x:v>Independent mission review confirmed exact issuance ancestry and allowed-path compliance; shared layout/routes/menu/footer/brand reuse; approved nine-section narrative; honest under-development language; four concentric rings labeled Value, Knowledge, Teams, and People with labels painted above rings; one olive thesis surface; distinct Organizations-specific mailto and general /contact/ actions; canonical header/footer order and correct header aria-current; no horizontal overflow at 390px or 1440px; mobile Enter/Escape/focus-return/nav-close/desktop-resize behavior; and no preview/export scaffolding. Full suite passed 9/9 in both root and /alaya-crafts-website base-path modes. Styled full-page captures at 1440px and 390px were independently reviewed.</x:v>
+      </x:c>
+      <x:c r="E29" s="9" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F29" s="9" t="str">
+        <x:v>None required. Keep the same page-specific gate and recurring regression checks for the remaining Ideas, launch article, and Contact migrations.</x:v>
+      </x:c>
+      <x:c r="G29" s="9" t="str">
+        <x:v>Fixed / Approved</x:v>
+      </x:c>
+      <x:c r="H29" s="9" t="str">
+        <x:v>Accepted by Codex disposition of AW-20260903-003. This closes the For Organizations portion of QA-CAND-004/005 only; no deployment or global gate closure.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="30" ht="18" customHeight="1"/>
     <x:row r="31" ht="18" customHeight="1"/>
     <x:row r="32" ht="18" customHeight="1"/>

</xml_diff>

<commit_message>
Close stale CIE regression hardening candidate
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R7fa8e4a562f5486d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R0233a0f9577f4b6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R58c1d4056dc947d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rda4d1526d3d04715"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R88a1de155c694168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="Rb8ea637bc14843d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,6 +1095,23 @@
         <x:v>ACCEPTED — For Organizations clears its page-specific Production Reference Gate; no push, merge, deployment, or broader product approval implied</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="120" customHeight="1">
+      <x:c r="A22" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="str">
+        <x:v>QA-CAND-003 preflight — proposed CIE diagram hardening already present</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="str">
+        <x:v>Before issuing a new mission, Codex checked the current CIE test and commit history. tests/cie-professional.spec.mjs already scrolls the capability diagram into view, samples the center of every strong label with document.elementFromPoint, rejects .diagram-path as the topmost element, and requires the sampled node to remain inside its card. Git blame traces this failure-sensitive assertion to bf9518a (Build production CIE Professional page). No implementation or test change was needed and no mission was issued.</x:v>
+      </x:c>
+      <x:c r="D22" s="9" t="str">
+        <x:v>0 — stale recommendation reconciled</x:v>
+      </x:c>
+      <x:c r="E22" s="9" t="str">
+        <x:v>CLOSED — requested regression hardening already exists; duplicate mission avoided</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2206,7 +2223,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="27" ht="18" customHeight="1">
+    <x:row r="27" ht="120" customHeight="1">
       <x:c r="A27" s="6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-09-03</x:t>
@@ -2232,20 +2249,14 @@
           <x:t xml:space="preserve">Note</x:t>
         </x:is>
       </x:c>
-      <x:c r="F27" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">None — fix confirmed holding in production. Recommend adding an elementFromPoint-style assertion to cie-professional.spec.mjs, since the current suite only checks .capability-diagram visibility, not label-on-top stacking — this is the second time this exact bug class has appeared on this exact page.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G27" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fixed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H27" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manual visual screenshot retained for this session as supporting evidence, not just DOM assertions.</x:t>
-        </x:is>
+      <x:c r="F27" s="6" t="str">
+        <x:v>None — current tests/cie-professional.spec.mjs already contains the recommended elementFromPoint label paint-order assertion.</x:v>
+      </x:c>
+      <x:c r="G27" s="6" t="str">
+        <x:v>Fixed / Covered by regression test</x:v>
+      </x:c>
+      <x:c r="H27" s="6" t="str">
+        <x:v>Reconciled 2026-09-03 during QA-CAND-003 issuance preflight. The assertion was already present in bf9518a; no new mission or code change was required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="120" customHeight="1">

</xml_diff>

<commit_message>
Accept Mission AW-20260903-004 and reconcile QA
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rda4d1526d3d04715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R88a1de155c694168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="Rb8ea637bc14843d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R027fd2687ce74360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="Rd44407fe93f74955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="Re5e0baa218c34010"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1112,6 +1112,23 @@
         <x:v>CLOSED — requested regression hardening already exists; duplicate mission avoided</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="135" customHeight="1">
+      <x:c r="A23" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B23" s="9" t="str">
+        <x:v>Mission AW-20260903-004 — Ideas index and launch article migration</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="str">
+        <x:v>Codex independently reviewed commit 34863f9 from exact issuance parent d0b323f. The commit stayed within the five authorized implementation paths plus claude-return.md. The Ideas index contains the approved six-part editorial structure and exactly one real launch item. The launch article preserves the complete approved title, metadata, 12 paragraphs, five section headings, and contextual CIE connection. Both routes consume the shared shell and identify Ideas as active. Full checked-in suites passed 16/16 in root mode and 16/16 with BASE_PATH=/alaya-crafts-website. Styled 1440px and 390px captures of both routes were reviewed for hierarchy, spacing, metadata, long-form reading measure, and responsive reflow.</x:v>
+      </x:c>
+      <x:c r="D23" s="9" t="str">
+        <x:v>0 new — no blocking or corrective findings</x:v>
+      </x:c>
+      <x:c r="E23" s="9" t="str">
+        <x:v>ACCEPTED — Ideas index and launch article clear their page-specific Production Reference Gate; Contact remains pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2321,7 +2338,32 @@
         <x:v>Accepted by Codex disposition of AW-20260903-003. This closes the For Organizations portion of QA-CAND-004/005 only; no deployment or global gate closure.</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="18" customHeight="1"/>
+    <x:row r="30" ht="140" customHeight="1">
+      <x:c r="A30" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B30" s="9" t="str">
+        <x:v>Production / Ideas index and launch article migration</x:v>
+      </x:c>
+      <x:c r="C30" s="9" t="str">
+        <x:v>src/pages/ideas.mjs + src/pages/idea-article.mjs + src/assets/ideas.css + generated dist/ideas routes</x:v>
+      </x:c>
+      <x:c r="D30" s="9" t="str">
+        <x:v>Independent mission review confirmed exact issuance ancestry and allowed-path compliance; shared shell reuse on both routes; approved six-part Ideas index; exactly one real Field Work item marked Developed and dated 27 August 2026; complete settled article body with five section headings and 12 reading paragraphs; correct article, Contact, CIE Professional, and return-to-Ideas destinations; canonical navigation and header aria-current; comfortable desktop reading measure; no horizontal overflow at 390px or 1440px; mobile keyboard/menu behavior; and no preview, inspector, document-toggle, or dependency scaffolding. Full suite passed 16/16 in both root and /alaya-crafts-website base-path modes. Both routes were visually reviewed at desktop and mobile widths.</x:v>
+      </x:c>
+      <x:c r="E30" s="9" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F30" s="9" t="str">
+        <x:v>None required. Preserve the existing editorial constraints and regression suite; proceed separately with the remaining Contact production migration.</x:v>
+      </x:c>
+      <x:c r="G30" s="9" t="str">
+        <x:v>Fixed / Approved</x:v>
+      </x:c>
+      <x:c r="H30" s="9" t="str">
+        <x:v>Accepted by Codex disposition of AW-20260903-004. This closes the Ideas and launch-article portion of QA-CAND-005 only; no deployment or publication-status change beyond the approved repository content.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="31" ht="18" customHeight="1"/>
     <x:row r="32" ht="18" customHeight="1"/>
     <x:row r="33" ht="18" customHeight="1"/>

</xml_diff>

<commit_message>
Accept Mission AW-20260903-005 and reconcile QA
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R027fd2687ce74360"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="Rd44407fe93f74955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="Re5e0baa218c34010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R750335e8606c407d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R4d50d366f2e64320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="Rebea87f8a9914938"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1129,6 +1129,23 @@
         <x:v>ACCEPTED — Ideas index and launch article clear their page-specific Production Reference Gate; Contact remains pending</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="135" customHeight="1">
+      <x:c r="A24" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B24" s="9" t="str">
+        <x:v>Mission AW-20260903-005 — Contact production migration</x:v>
+      </x:c>
+      <x:c r="C24" s="9" t="str">
+        <x:v>Codex independently reviewed commit 10c0866 from exact issuance parent 97571ca. The commit stayed within the four authorized implementation paths plus claude-return.md. The Contact route uses the shared shell, preserves the approved compact two-column-to-one-column composition and exact direct-human-contact copy, exposes curious@alayacrafts.com as the sole visible contact mechanism, and adds no form, scheduler, phone, social, tracking, or response-time promise. Existing Homepage, Organizations, and Ideas invitations resolve to the canonical Contact route. Full checked-in suites passed 22/22 in root mode and 22/22 with BASE_PATH=/alaya-crafts-website. Esteban confirmed curious@alayacrafts.com as the correct official address before acceptance.</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="str">
+        <x:v>0 new — no blocking or corrective findings</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="str">
+        <x:v>ACCEPTED — Contact clears its page-specific Production Reference Gate; all approved V1 routes now have accepted production implementations</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2364,7 +2381,32 @@
         <x:v>Accepted by Codex disposition of AW-20260903-004. This closes the Ideas and launch-article portion of QA-CAND-005 only; no deployment or publication-status change beyond the approved repository content.</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="18" customHeight="1"/>
+    <x:row r="31" ht="140" customHeight="1">
+      <x:c r="A31" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B31" s="9" t="str">
+        <x:v>Production / Contact migration</x:v>
+      </x:c>
+      <x:c r="C31" s="9" t="str">
+        <x:v>src/pages/contact.mjs + src/assets/contact.css + generated dist/contact/index.html</x:v>
+      </x:c>
+      <x:c r="D31" s="9" t="str">
+        <x:v>Independent mission review confirmed exact issuance ancestry and allowed-path compliance; shared shell reuse; exact approved Contact copy; curious@alayacrafts.com as the only visible and usable contact mechanism; no form, fields, phone, scheduler, social channel, tracking, service offer, or response-time promise; canonical header/footer order and Contact active state; compact responsive composition; inbound Contact links from Homepage, Organizations, and Ideas; zero horizontal overflow at 390px and 1440px; mobile keyboard/menu behavior; and no preview, inspector, dependency, iframe, or embedded-raster scaffolding. Full suite passed 22/22 in both root and /alaya-crafts-website base-path modes. Esteban explicitly confirmed the official address before acceptance.</x:v>
+      </x:c>
+      <x:c r="E31" s="9" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F31" s="9" t="str">
+        <x:v>None required. Retain the Contact and shared-shell regression assertions in the full suite.</x:v>
+      </x:c>
+      <x:c r="G31" s="9" t="str">
+        <x:v>Fixed / Approved</x:v>
+      </x:c>
+      <x:c r="H31" s="9" t="str">
+        <x:v>Accepted by Codex disposition of AW-20260903-005. This closes the Contact portions of QA-CAND-004 and QA-CAND-005; no push, merge, deployment, or broader product change is implied.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="32" ht="18" customHeight="1"/>
     <x:row r="33" ht="18" customHeight="1"/>
     <x:row r="34" ht="18" customHeight="1"/>

</xml_diff>

<commit_message>
Accept Mission AW-20260903-006 and record release readiness
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R750335e8606c407d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R4d50d366f2e64320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="Rebea87f8a9914938"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R301ef5077a924e50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R026ade9e7c7643ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R3def43ac2d2d4dbd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1146,6 +1146,23 @@
         <x:v>ACCEPTED — Contact clears its page-specific Production Reference Gate; all approved V1 routes now have accepted production implementations</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="145" customHeight="1">
+      <x:c r="A25" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B25" s="9" t="str">
+        <x:v>Mission AW-20260903-006 — release and deployment readiness verification</x:v>
+      </x:c>
+      <x:c r="C25" s="9" t="str">
+        <x:v>Codex independently accepted the verification-only return at f3b7a2d from exact issuance parent fa68576. The return commit added only claude-return.md. The integrated site passed 22/22 tests in root mode and 22/22 with BASE_PATH=/alaya-crafts-website. The pre-return unpublished range contains 19 linear, single-parent commits, all accounted for by mission control, accepted page work, and governed QA. Both generated artifacts contain the six ADR routes with working local references. The workflow definition correctly gates the Pages artifact and deploy job on the base-path build and test. QA-CAND-001 links resolve in both modes and remain a non-blocking maintainability note.</x:v>
+      </x:c>
+      <x:c r="D25" s="9" t="str">
+        <x:v>0 new defects — 1 publication prerequisite and external checks remain</x:v>
+      </x:c>
+      <x:c r="E25" s="9" t="str">
+        <x:v>ACCEPTED — locally release-ready; not published. Owner authorization to push and external GitHub Pages settings checks remain separate steps</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2407,7 +2424,32 @@
         <x:v>Accepted by Codex disposition of AW-20260903-005. This closes the Contact portions of QA-CAND-004 and QA-CAND-005; no push, merge, deployment, or broader product change is implied.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="18" customHeight="1"/>
+    <x:row r="32" ht="155" customHeight="1">
+      <x:c r="A32" s="9" t="str">
+        <x:v>2026-09-03</x:v>
+      </x:c>
+      <x:c r="B32" s="9" t="str">
+        <x:v>Release / integrated repository readiness</x:v>
+      </x:c>
+      <x:c r="C32" s="9" t="str">
+        <x:v>main at fa68576 pre-return + generated dist/ + .github/workflows/pages.yml</x:v>
+      </x:c>
+      <x:c r="D32" s="9" t="str">
+        <x:v>Independent review confirmed clean and linear local history; 19 pre-return commits ahead of the cached origin/main ref; no unexpected merge, tracked generated output, unexplained binary, or secret-like changed content; reproducible dependency install; exact six-route artifact in both supported modes; zero broken local references reported by the verification actor; QA-CAND-001 body links resolving in both modes; and a Pages workflow that builds and tests the project-site base path before artifact upload and deployment. Codex independently reran the complete suite: 22/22 passed in root mode and 22/22 in repository-base-path mode.</x:v>
+      </x:c>
+      <x:c r="E32" s="9" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F32" s="9" t="str">
+        <x:v>Do not call the site published yet. Obtain Esteban's explicit authorization before pushing local main. After the push, verify the GitHub Pages workflow and configured Pages environment externally. Canonical-domain/DNS and mailbox delivery remain separate external checks if they are part of the intended launch.</x:v>
+      </x:c>
+      <x:c r="G32" s="9" t="str">
+        <x:v>Ready locally / Not published</x:v>
+      </x:c>
+      <x:c r="H32" s="9" t="str">
+        <x:v>Accepted by Codex disposition of AW-20260903-006. Local source, build, tests, artifacts, routing, and workflow definition are ready. Publication state remains not ready solely because the accepted commits have not been pushed; external hosting settings were outside mission authority.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="33" ht="18" customHeight="1"/>
     <x:row r="34" ht="18" customHeight="1"/>
     <x:row r="35" ht="18" customHeight="1"/>

</xml_diff>

<commit_message>
Accept Mission AW-20260904-002 visual refinements
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R301ef5077a924e50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R026ade9e7c7643ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R3def43ac2d2d4dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R191985ec7e774a70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="Rd0324a0e86954187"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R4a506d307b0741da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1163,6 +1163,23 @@
         <x:v>ACCEPTED — locally release-ready; not published. Owner authorization to push and external GitHub Pages settings checks remain separate steps</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="145" customHeight="1">
+      <x:c r="A26" s="9" t="str">
+        <x:v>2026-09-04</x:v>
+      </x:c>
+      <x:c r="B26" s="9" t="str">
+        <x:v>Mission AW-20260904-002 — Homepage Section 05 and Section 07 visual refinement</x:v>
+      </x:c>
+      <x:c r="C26" s="9" t="str">
+        <x:v>Codex independently accepted the implementation at 9d2ef46 from exact issuance parent fd8657b. Section 05 now uses one code-native capability landscape that maps terrain, knowledge contours, a technology connection path, visible intelligence relationships, and cultivation marks. Section 07 now shows a recognizable layered mountain landscape. The approved visible copy and product boundaries remain unchanged. Desktop and 390px visual review found no clipping or horizontal overflow. The complete suite passed 25/25 in root mode and 25/25 with BASE_PATH=/alaya-crafts-website.</x:v>
+      </x:c>
+      <x:c r="D26" s="9" t="str">
+        <x:v>0 new defects</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="str">
+        <x:v>ACCEPTED — visual refinement complete; no push or deployment performed</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2450,7 +2467,32 @@
         <x:v>Accepted by Codex disposition of AW-20260903-006. Local source, build, tests, artifacts, routing, and workflow definition are ready. Publication state remains not ready solely because the accepted commits have not been pushed; external hosting settings were outside mission authority.</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="18" customHeight="1"/>
+    <x:row r="33" ht="155" customHeight="1">
+      <x:c r="A33" s="9" t="str">
+        <x:v>2026-09-04</x:v>
+      </x:c>
+      <x:c r="B33" s="9" t="str">
+        <x:v>Homepage visual refinement — Sections 05 and 07</x:v>
+      </x:c>
+      <x:c r="C33" s="9" t="str">
+        <x:v>src/pages/home.mjs + src/assets/home.css + tests/homepage.spec.mjs</x:v>
+      </x:c>
+      <x:c r="D33" s="9" t="str">
+        <x:v>Section 05 replaces decorative arcs with a single meaningful landscape: capability terrain, knowledge contours, technology connection path, intelligence relationship lines, and cultivation marks. Section 07 replaces the abstract semicircle with a recognizable layered mountain scene. Both are code-native inline SVG, decorative to assistive technology, and contain no fabricated product UI or data. Codex independently reviewed desktop and 390px rendering and reran both complete test modes: 25/25 passed in each.</x:v>
+      </x:c>
+      <x:c r="E33" s="9" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F33" s="9" t="str">
+        <x:v>Retain the current visual semantics, approved visible copy, responsive no-overflow behavior, and no-fabricated-product-UI boundary in future Homepage changes.</x:v>
+      </x:c>
+      <x:c r="G33" s="9" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="H33" s="9" t="str">
+        <x:v>Accepted by Codex disposition of AW-20260904-002 at 9d2ef46. Mission AW-20260904-001 remains superseded and was not executed. No push or deployment occurred in this mission.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="34" ht="18" customHeight="1"/>
     <x:row r="35" ht="18" customHeight="1"/>
     <x:row r="36" ht="18" customHeight="1"/>

</xml_diff>

<commit_message>
Accept Mission AW-20260904-004 artwork and favicon
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R191985ec7e774a70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="Rd0324a0e86954187"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R4a506d307b0741da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R98b3f47ecc5a4ac5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="Re039b5dfe7044ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R184c79a0fb324c3f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1180,6 +1180,23 @@
         <x:v>ACCEPTED — visual refinement complete; no push or deployment performed</x:v>
       </x:c>
     </x:row>
+    <x:row r="27" ht="150" customHeight="1">
+      <x:c r="A27" s="9" t="str">
+        <x:v>2026-09-04</x:v>
+      </x:c>
+      <x:c r="B27" s="9" t="str">
+        <x:v>Mission AW-20260904-004 — approved Homepage artwork and favicon</x:v>
+      </x:c>
+      <x:c r="C27" s="9" t="str">
+        <x:v>Codex independently accepted the implementation at f2eb249 from exact issuance parent e91f10b. The three Esteban-supplied SVGs remain byte-identical to their immutable mission inputs. Section 05 selects the approved desktop or mobile composition at the existing breakpoint; Section 07 uses the approved atmospheric horizon asset at both widths. All six routes receive one shared SVG favicon derived from the existing Alaya header mark. Desktop and 390px visual review confirmed correct composition, label placement, proportional horizon rendering, no horizontal overflow, and a clear 32px favicon. Both complete suites passed 29/29.</x:v>
+      </x:c>
+      <x:c r="D27" s="9" t="str">
+        <x:v>0 new defects</x:v>
+      </x:c>
+      <x:c r="E27" s="9" t="str">
+        <x:v>ACCEPTED — artwork and favicon ready locally; no push or deployment performed</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2493,7 +2510,32 @@
         <x:v>Accepted by Codex disposition of AW-20260904-002 at 9d2ef46. Mission AW-20260904-001 remains superseded and was not executed. No push or deployment occurred in this mission.</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="18" customHeight="1"/>
+    <x:row r="34" ht="160" customHeight="1">
+      <x:c r="A34" s="9" t="str">
+        <x:v>2026-09-04</x:v>
+      </x:c>
+      <x:c r="B34" s="9" t="str">
+        <x:v>Homepage approved artwork and shared favicon</x:v>
+      </x:c>
+      <x:c r="C34" s="9" t="str">
+        <x:v>src/assets/alaya-05-*.svg + src/assets/alaya-07-horizon.svg + src/assets/favicon.svg + Homepage/shared layout</x:v>
+      </x:c>
+      <x:c r="D34" s="9" t="str">
+        <x:v>Section 05 now uses the approved, separately composed desktop and mobile SVGs; Section 07 uses the approved atmospheric horizon SVG without geometric stretching. The three deployable artwork files are byte-identical to the governed mission inputs and retain their content credentials. Every generated route has exactly one correctly resolved SVG favicon based on the existing Alaya header mark. Codex independently reviewed 1440px and 390px rendering and reran both full deployment modes: 29/29 passed in each.</x:v>
+      </x:c>
+      <x:c r="E34" s="9" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F34" s="9" t="str">
+        <x:v>Retain the supplied artwork hashes, responsive Section 05 selection, proportional Section 07 crop, shared favicon routing, visible copy, and no-overflow behavior in future changes.</x:v>
+      </x:c>
+      <x:c r="G34" s="9" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="H34" s="9" t="str">
+        <x:v>Accepted by Codex disposition of AW-20260904-004 at f2eb249. AW-20260904-003 remains superseded without execution. No push or deployment occurred under this mission.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="35" ht="18" customHeight="1"/>
     <x:row r="36" ht="18" customHeight="1"/>
     <x:row r="37" ht="18" customHeight="1"/>

</xml_diff>

<commit_message>
Accept mission AW-20260904-005 custom-domain correction
</commit_message>
<xml_diff>
--- a/reviews/qa/Alaya_Website_QA_Tracker.xlsx
+++ b/reviews/qa/Alaya_Website_QA_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R98b3f47ecc5a4ac5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="Re039b5dfe7044ab4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R184c79a0fb324c3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R759f463e05174d2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session History" sheetId="2" r:id="R7c80c03efec24de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Log" sheetId="3" r:id="R4fb68172a19b40cc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1197,6 +1197,23 @@
         <x:v>ACCEPTED — artwork and favicon ready locally; no push or deployment performed</x:v>
       </x:c>
     </x:row>
+    <x:row r="28" ht="145" customHeight="1">
+      <x:c r="A28" s="9" t="str">
+        <x:v>2026-09-04</x:v>
+      </x:c>
+      <x:c r="B28" s="9" t="str">
+        <x:v>Mission AW-20260904-005 — custom-domain root-path deployment correction</x:v>
+      </x:c>
+      <x:c r="C28" s="9" t="str">
+        <x:v>Codex independently accepted implementation b51db15 from exact issuance parent 8a160f7. The Pages workflow now proves both root and repository-subpath modes, then performs a final root-mode build immediately before artifact upload. Both complete suites passed 29/29. The final dist contains no /alaya-crafts-website/ references and includes the shared CSS, favicon, and all six routes required for alayacrafts.com.</x:v>
+      </x:c>
+      <x:c r="D28" s="9" t="str">
+        <x:v>0 new defects</x:v>
+      </x:c>
+      <x:c r="E28" s="9" t="str">
+        <x:v>ACCEPTED — root-path deployment artifact ready for authorized publication</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2536,7 +2553,32 @@
         <x:v>Accepted by Codex disposition of AW-20260904-004 at f2eb249. AW-20260904-003 remains superseded without execution. No push or deployment occurred under this mission.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="18" customHeight="1"/>
+    <x:row r="35" ht="155" customHeight="1">
+      <x:c r="A35" s="9" t="str">
+        <x:v>2026-09-04</x:v>
+      </x:c>
+      <x:c r="B35" s="9" t="str">
+        <x:v>Custom-domain root-path deployment artifact</x:v>
+      </x:c>
+      <x:c r="C35" s="9" t="str">
+        <x:v>.github/workflows/pages.yml + generated dist validation</x:v>
+      </x:c>
+      <x:c r="D35" s="9" t="str">
+        <x:v>The deployment workflow runs the root suite, the /alaya-crafts-website compatibility suite, and then a fresh root build as the exact artifact uploaded to GitHub Pages. Independent verification passed 29/29 in both modes; the final artifact has root-relative URLs, no repository-path prefix, and contains the favicon, shared stylesheet, Homepage, CIE Professional, For Organizations, Ideas, article, and Contact outputs.</x:v>
+      </x:c>
+      <x:c r="E35" s="9" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F35" s="9" t="str">
+        <x:v>Retain the final root build immediately before upload and both deployment-mode test runs. Verify the apex domain, www redirect, route assets, and HTTPS after publication.</x:v>
+      </x:c>
+      <x:c r="G35" s="9" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="H35" s="9" t="str">
+        <x:v>Accepted by Codex disposition of AW-20260904-005 at b51db15. Actor scope was limited to the workflow and its return artifact; DNS, repository settings, push, and live publication remain separate authorized operator actions.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="36" ht="18" customHeight="1"/>
     <x:row r="37" ht="18" customHeight="1"/>
     <x:row r="38" ht="18" customHeight="1"/>

</xml_diff>